<commit_message>
roud up GPT-4o base acc and update p-values to adjusted
</commit_message>
<xml_diff>
--- a/eval/learning-curve/results/statistical_tests_full150.xlsx
+++ b/eval/learning-curve/results/statistical_tests_full150.xlsx
@@ -518,7 +518,7 @@
         <v>0.102</v>
       </c>
       <c r="J2" t="n">
-        <v>0.293</v>
+        <v>0.319</v>
       </c>
     </row>
     <row r="3">
@@ -558,7 +558,7 @@
         <v>0.102</v>
       </c>
       <c r="J3" t="n">
-        <v>0.33</v>
+        <v>0.334</v>
       </c>
     </row>
     <row r="4">
@@ -598,7 +598,7 @@
         <v>0.169</v>
       </c>
       <c r="J4" t="n">
-        <v>0.594</v>
+        <v>0.681</v>
       </c>
     </row>
     <row r="5">
@@ -678,7 +678,7 @@
         <v>0.0877</v>
       </c>
       <c r="J6" t="n">
-        <v>0.48</v>
+        <v>0.5570000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -718,7 +718,7 @@
         <v>0.0877</v>
       </c>
       <c r="J7" t="n">
-        <v>0.453</v>
+        <v>0.495</v>
       </c>
     </row>
     <row r="8">
@@ -758,7 +758,7 @@
         <v>0.156</v>
       </c>
       <c r="J8" t="n">
-        <v>0.647</v>
+        <v>0.755</v>
       </c>
     </row>
     <row r="9">
@@ -798,7 +798,7 @@
         <v>0.156</v>
       </c>
       <c r="J9" t="n">
-        <v>0.732</v>
+        <v>0.765</v>
       </c>
     </row>
     <row r="10">
@@ -838,7 +838,7 @@
         <v>0.167</v>
       </c>
       <c r="J10" t="n">
-        <v>0.555</v>
+        <v>0.651</v>
       </c>
     </row>
     <row r="11">
@@ -878,7 +878,7 @@
         <v>0.167</v>
       </c>
       <c r="J11" t="n">
-        <v>0.732</v>
+        <v>0.773</v>
       </c>
     </row>
     <row r="12">
@@ -918,7 +918,7 @@
         <v>0.152</v>
       </c>
       <c r="J12" t="n">
-        <v>0.628</v>
+        <v>0.725</v>
       </c>
     </row>
     <row r="13">
@@ -998,7 +998,7 @@
         <v>0.0829</v>
       </c>
       <c r="J14" t="n">
-        <v>0.214</v>
+        <v>0.251</v>
       </c>
     </row>
     <row r="15">
@@ -1038,7 +1038,7 @@
         <v>0.0829</v>
       </c>
       <c r="J15" t="n">
-        <v>0.33</v>
+        <v>0.308</v>
       </c>
     </row>
     <row r="16">
@@ -1078,7 +1078,7 @@
         <v>0.174</v>
       </c>
       <c r="J16" t="n">
-        <v>0.653</v>
+        <v>0.768</v>
       </c>
     </row>
     <row r="17">
@@ -1118,7 +1118,7 @@
         <v>0.174</v>
       </c>
       <c r="J17" t="n">
-        <v>0.732</v>
+        <v>0.765</v>
       </c>
     </row>
     <row r="18">
@@ -1158,7 +1158,7 @@
         <v>0.07190000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>0.015</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="19">
@@ -1198,7 +1198,7 @@
         <v>0.07190000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>0.014</v>
+        <v>0.0372</v>
       </c>
     </row>
     <row r="20">
@@ -1238,7 +1238,7 @@
         <v>0.0842</v>
       </c>
       <c r="J20" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.08890000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -1278,7 +1278,7 @@
         <v>0.0842</v>
       </c>
       <c r="J21" t="n">
-        <v>0.0997</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="22">
@@ -1318,7 +1318,7 @@
         <v>0.165</v>
       </c>
       <c r="J22" t="n">
-        <v>0.111</v>
+        <v>0.126</v>
       </c>
     </row>
     <row r="23">
@@ -1358,7 +1358,7 @@
         <v>0.165</v>
       </c>
       <c r="J23" t="n">
-        <v>0.0997</v>
+        <v>0.123</v>
       </c>
     </row>
     <row r="24">
@@ -1398,7 +1398,7 @@
         <v>0.175</v>
       </c>
       <c r="J24" t="n">
-        <v>0.366</v>
+        <v>0.395</v>
       </c>
     </row>
     <row r="25">
@@ -1438,7 +1438,7 @@
         <v>0.175</v>
       </c>
       <c r="J25" t="n">
-        <v>0.33</v>
+        <v>0.323</v>
       </c>
     </row>
     <row r="26">
@@ -1478,7 +1478,7 @@
         <v>0.175</v>
       </c>
       <c r="J26" t="n">
-        <v>0.435</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="27">
@@ -1518,7 +1518,7 @@
         <v>0.175</v>
       </c>
       <c r="J27" t="n">
-        <v>0.453</v>
+        <v>0.495</v>
       </c>
     </row>
     <row r="28">
@@ -1558,7 +1558,7 @@
         <v>0.19</v>
       </c>
       <c r="J28" t="n">
-        <v>0.54</v>
+        <v>0.617</v>
       </c>
     </row>
     <row r="29">
@@ -1598,7 +1598,7 @@
         <v>0.19</v>
       </c>
       <c r="J29" t="n">
-        <v>0.508</v>
+        <v>0.598</v>
       </c>
     </row>
     <row r="30">
@@ -1638,7 +1638,7 @@
         <v>0.0931</v>
       </c>
       <c r="J30" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.08890000000000001</v>
       </c>
     </row>
     <row r="31">
@@ -1678,7 +1678,7 @@
         <v>0.0931</v>
       </c>
       <c r="J31" t="n">
-        <v>0.014</v>
+        <v>0.0372</v>
       </c>
     </row>
     <row r="32">
@@ -1718,7 +1718,7 @@
         <v>0.12</v>
       </c>
       <c r="J32" t="n">
-        <v>0.886</v>
+        <v>0.903</v>
       </c>
     </row>
     <row r="33">
@@ -1758,7 +1758,7 @@
         <v>0.12</v>
       </c>
       <c r="J33" t="n">
-        <v>0.575</v>
+        <v>0.634</v>
       </c>
     </row>
     <row r="34">
@@ -1798,7 +1798,7 @@
         <v>0.249</v>
       </c>
       <c r="J34" t="n">
-        <v>0.445</v>
+        <v>0.271</v>
       </c>
     </row>
     <row r="35">
@@ -1878,7 +1878,7 @@
         <v>0.134</v>
       </c>
       <c r="J36" t="n">
-        <v>0.886</v>
+        <v>0.768</v>
       </c>
     </row>
     <row r="37">
@@ -1918,7 +1918,7 @@
         <v>0.134</v>
       </c>
       <c r="J37" t="n">
-        <v>0.575</v>
+        <v>0.622</v>
       </c>
     </row>
     <row r="38">
@@ -1958,7 +1958,7 @@
         <v>0.22</v>
       </c>
       <c r="J38" t="n">
-        <v>0.664</v>
+        <v>0.581</v>
       </c>
     </row>
     <row r="39">
@@ -1998,7 +1998,7 @@
         <v>0.22</v>
       </c>
       <c r="J39" t="n">
-        <v>0.495</v>
+        <v>0.447</v>
       </c>
     </row>
     <row r="40">
@@ -2038,7 +2038,7 @@
         <v>0.185</v>
       </c>
       <c r="J40" t="n">
-        <v>0.445</v>
+        <v>0.395</v>
       </c>
     </row>
     <row r="41">
@@ -2078,7 +2078,7 @@
         <v>0.185</v>
       </c>
       <c r="J41" t="n">
-        <v>0.24</v>
+        <v>0.179</v>
       </c>
     </row>
     <row r="42">
@@ -2118,7 +2118,7 @@
         <v>0.255</v>
       </c>
       <c r="J42" t="n">
-        <v>0.445</v>
+        <v>0.395</v>
       </c>
     </row>
     <row r="43">
@@ -2158,7 +2158,7 @@
         <v>0.255</v>
       </c>
       <c r="J43" t="n">
-        <v>0.495</v>
+        <v>0.362</v>
       </c>
     </row>
     <row r="44">
@@ -2198,7 +2198,7 @@
         <v>0.107</v>
       </c>
       <c r="J44" t="n">
-        <v>0.886</v>
+        <v>0.829</v>
       </c>
     </row>
     <row r="45">
@@ -2238,7 +2238,7 @@
         <v>0.107</v>
       </c>
       <c r="J45" t="n">
-        <v>0.575</v>
+        <v>0.642</v>
       </c>
     </row>
     <row r="46">
@@ -2278,7 +2278,7 @@
         <v>0.224</v>
       </c>
       <c r="J46" t="n">
-        <v>0.445</v>
+        <v>0.396</v>
       </c>
     </row>
     <row r="47">
@@ -2318,7 +2318,7 @@
         <v>0.224</v>
       </c>
       <c r="J47" t="n">
-        <v>0.277</v>
+        <v>0.222</v>
       </c>
     </row>
     <row r="48">
@@ -2358,7 +2358,7 @@
         <v>0.0584</v>
       </c>
       <c r="J48" t="n">
-        <v>0.445</v>
+        <v>0.285</v>
       </c>
     </row>
     <row r="49">
@@ -2398,7 +2398,7 @@
         <v>0.0584</v>
       </c>
       <c r="J49" t="n">
-        <v>0.495</v>
+        <v>0.442</v>
       </c>
     </row>
     <row r="50">
@@ -2438,7 +2438,7 @@
         <v>0.11</v>
       </c>
       <c r="J50" t="n">
-        <v>0.886</v>
+        <v>0.883</v>
       </c>
     </row>
     <row r="51">
@@ -2478,7 +2478,7 @@
         <v>0.11</v>
       </c>
       <c r="J51" t="n">
-        <v>0.575</v>
+        <v>0.642</v>
       </c>
     </row>
     <row r="52">
@@ -2518,7 +2518,7 @@
         <v>0.195</v>
       </c>
       <c r="J52" t="n">
-        <v>0.776</v>
+        <v>0.651</v>
       </c>
     </row>
     <row r="53">
@@ -2558,7 +2558,7 @@
         <v>0.195</v>
       </c>
       <c r="J53" t="n">
-        <v>0.575</v>
+        <v>0.622</v>
       </c>
     </row>
     <row r="54">
@@ -2598,7 +2598,7 @@
         <v>0.183</v>
       </c>
       <c r="J54" t="n">
-        <v>0.886</v>
+        <v>0.917</v>
       </c>
     </row>
     <row r="55">
@@ -2638,7 +2638,7 @@
         <v>0.183</v>
       </c>
       <c r="J55" t="n">
-        <v>0.744</v>
+        <v>0.827</v>
       </c>
     </row>
     <row r="56">
@@ -2678,7 +2678,7 @@
         <v>0.189</v>
       </c>
       <c r="J56" t="n">
-        <v>0.886</v>
+        <v>0.829</v>
       </c>
     </row>
     <row r="57">
@@ -2718,7 +2718,7 @@
         <v>0.189</v>
       </c>
       <c r="J57" t="n">
-        <v>0.696</v>
+        <v>0.765</v>
       </c>
     </row>
     <row r="58">
@@ -2758,7 +2758,7 @@
         <v>0.195</v>
       </c>
       <c r="J58" t="n">
-        <v>0.886</v>
+        <v>0.829</v>
       </c>
     </row>
     <row r="59">
@@ -2798,7 +2798,7 @@
         <v>0.195</v>
       </c>
       <c r="J59" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.765</v>
       </c>
     </row>
     <row r="60">
@@ -2838,7 +2838,7 @@
         <v>0.0954</v>
       </c>
       <c r="J60" t="n">
-        <v>0.0134</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="61">
@@ -2878,7 +2878,7 @@
         <v>0.0954</v>
       </c>
       <c r="J61" t="n">
-        <v>0.0148</v>
+        <v>0.0372</v>
       </c>
     </row>
     <row r="62">
@@ -2918,7 +2918,7 @@
         <v>0.186</v>
       </c>
       <c r="J62" t="n">
-        <v>0.45</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="63">
@@ -2958,7 +2958,7 @@
         <v>0.186</v>
       </c>
       <c r="J63" t="n">
-        <v>0.232</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="64">
@@ -3038,7 +3038,7 @@
         <v>0.266</v>
       </c>
       <c r="J65" t="n">
-        <v>0.233</v>
+        <v>0.323</v>
       </c>
     </row>
     <row r="66">
@@ -3078,7 +3078,7 @@
         <v>0.149</v>
       </c>
       <c r="J66" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.755</v>
       </c>
     </row>
     <row r="67">
@@ -3118,7 +3118,7 @@
         <v>0.149</v>
       </c>
       <c r="J67" t="n">
-        <v>0.749</v>
+        <v>0.765</v>
       </c>
     </row>
     <row r="68">
@@ -3158,7 +3158,7 @@
         <v>0.239</v>
       </c>
       <c r="J68" t="n">
-        <v>0.61</v>
+        <v>0.681</v>
       </c>
     </row>
     <row r="69">
@@ -3238,7 +3238,7 @@
         <v>0.148</v>
       </c>
       <c r="J70" t="n">
-        <v>0.61</v>
+        <v>0.669</v>
       </c>
     </row>
     <row r="71">
@@ -3278,7 +3278,7 @@
         <v>0.148</v>
       </c>
       <c r="J71" t="n">
-        <v>0.541</v>
+        <v>0.634</v>
       </c>
     </row>
     <row r="72">
@@ -3318,7 +3318,7 @@
         <v>0.267</v>
       </c>
       <c r="J72" t="n">
-        <v>0.61</v>
+        <v>0.681</v>
       </c>
     </row>
     <row r="73">
@@ -3358,7 +3358,7 @@
         <v>0.267</v>
       </c>
       <c r="J73" t="n">
-        <v>0.921</v>
+        <v>0.895</v>
       </c>
     </row>
     <row r="74">
@@ -3398,7 +3398,7 @@
         <v>0.144</v>
       </c>
       <c r="J74" t="n">
-        <v>0.249</v>
+        <v>0.347</v>
       </c>
     </row>
     <row r="75">
@@ -3438,7 +3438,7 @@
         <v>0.144</v>
       </c>
       <c r="J75" t="n">
-        <v>0.232</v>
+        <v>0.308</v>
       </c>
     </row>
     <row r="76">
@@ -3478,7 +3478,7 @@
         <v>0.264</v>
       </c>
       <c r="J76" t="n">
-        <v>0.983</v>
+        <v>0.9330000000000001</v>
       </c>
     </row>
     <row r="77">
@@ -3518,7 +3518,7 @@
         <v>0.264</v>
       </c>
       <c r="J77" t="n">
-        <v>0.495</v>
+        <v>0.622</v>
       </c>
     </row>
     <row r="78">
@@ -3558,7 +3558,7 @@
         <v>0.137</v>
       </c>
       <c r="J78" t="n">
-        <v>0.0585</v>
+        <v>0.08890000000000001</v>
       </c>
     </row>
     <row r="79">
@@ -3598,7 +3598,7 @@
         <v>0.137</v>
       </c>
       <c r="J79" t="n">
-        <v>0.055</v>
+        <v>0.066</v>
       </c>
     </row>
     <row r="80">
@@ -3638,7 +3638,7 @@
         <v>0.185</v>
       </c>
       <c r="J80" t="n">
-        <v>0.236</v>
+        <v>0.314</v>
       </c>
     </row>
     <row r="81">
@@ -3678,7 +3678,7 @@
         <v>0.185</v>
       </c>
       <c r="J81" t="n">
-        <v>0.232</v>
+        <v>0.308</v>
       </c>
     </row>
     <row r="82">
@@ -3718,7 +3718,7 @@
         <v>0.18</v>
       </c>
       <c r="J82" t="n">
-        <v>0.0597</v>
+        <v>0.09950000000000001</v>
       </c>
     </row>
     <row r="83">
@@ -3758,7 +3758,7 @@
         <v>0.18</v>
       </c>
       <c r="J83" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="84">
@@ -3838,7 +3838,7 @@
         <v>0.16</v>
       </c>
       <c r="J85" t="n">
-        <v>0.055</v>
+        <v>0.0572</v>
       </c>
     </row>
     <row r="86">
@@ -3878,7 +3878,7 @@
         <v>0.155</v>
       </c>
       <c r="J86" t="n">
-        <v>0.0597</v>
+        <v>0.08890000000000001</v>
       </c>
     </row>
     <row r="87">
@@ -3918,7 +3918,7 @@
         <v>0.155</v>
       </c>
       <c r="J87" t="n">
-        <v>0.0746</v>
+        <v>0.109</v>
       </c>
     </row>
     <row r="88">
@@ -3958,7 +3958,7 @@
         <v>0.162</v>
       </c>
       <c r="J88" t="n">
-        <v>0.0585</v>
+        <v>0.08890000000000001</v>
       </c>
     </row>
     <row r="89">
@@ -3998,7 +3998,7 @@
         <v>0.162</v>
       </c>
       <c r="J89" t="n">
-        <v>0.055</v>
+        <v>0.0572</v>
       </c>
     </row>
     <row r="90">
@@ -4038,7 +4038,7 @@
         <v>0.163</v>
       </c>
       <c r="J90" t="n">
-        <v>0.236</v>
+        <v>0.314</v>
       </c>
     </row>
     <row r="91">
@@ -4078,7 +4078,7 @@
         <v>0.163</v>
       </c>
       <c r="J91" t="n">
-        <v>0.234</v>
+        <v>0.334</v>
       </c>
     </row>
     <row r="92">
@@ -4118,7 +4118,7 @@
         <v>0.139</v>
       </c>
       <c r="J92" t="n">
-        <v>0.648</v>
+        <v>0.733</v>
       </c>
     </row>
     <row r="93">
@@ -4158,7 +4158,7 @@
         <v>0.139</v>
       </c>
       <c r="J93" t="n">
-        <v>0.673</v>
+        <v>0.622</v>
       </c>
     </row>
     <row r="94">
@@ -4198,7 +4198,7 @@
         <v>0.247</v>
       </c>
       <c r="J94" t="n">
-        <v>0.577</v>
+        <v>0.651</v>
       </c>
     </row>
     <row r="95">
@@ -4238,7 +4238,7 @@
         <v>0.247</v>
       </c>
       <c r="J95" t="n">
-        <v>0.865</v>
+        <v>0.895</v>
       </c>
     </row>
     <row r="96">
@@ -4278,7 +4278,7 @@
         <v>0.116</v>
       </c>
       <c r="J96" t="n">
-        <v>0.848</v>
+        <v>0.903</v>
       </c>
     </row>
     <row r="97">
@@ -4318,7 +4318,7 @@
         <v>0.116</v>
       </c>
       <c r="J97" t="n">
-        <v>0.865</v>
+        <v>0.895</v>
       </c>
     </row>
     <row r="98">
@@ -4358,7 +4358,7 @@
         <v>0.224</v>
       </c>
       <c r="J98" t="n">
-        <v>0.577</v>
+        <v>0.651</v>
       </c>
     </row>
     <row r="99">
@@ -4398,7 +4398,7 @@
         <v>0.224</v>
       </c>
       <c r="J99" t="n">
-        <v>0.865</v>
+        <v>0.895</v>
       </c>
     </row>
     <row r="100">
@@ -4438,7 +4438,7 @@
         <v>0.152</v>
       </c>
       <c r="J100" t="n">
-        <v>0.694</v>
+        <v>0.768</v>
       </c>
     </row>
     <row r="101">
@@ -4478,7 +4478,7 @@
         <v>0.152</v>
       </c>
       <c r="J101" t="n">
-        <v>0.836</v>
+        <v>0.765</v>
       </c>
     </row>
     <row r="102">
@@ -4518,7 +4518,7 @@
         <v>0.256</v>
       </c>
       <c r="J102" t="n">
-        <v>0.577</v>
+        <v>0.616</v>
       </c>
     </row>
     <row r="103">
@@ -4558,7 +4558,7 @@
         <v>0.256</v>
       </c>
       <c r="J103" t="n">
-        <v>0.836</v>
+        <v>0.765</v>
       </c>
     </row>
     <row r="104">
@@ -4598,7 +4598,7 @@
         <v>0.107</v>
       </c>
       <c r="J104" t="n">
-        <v>0.577</v>
+        <v>0.616</v>
       </c>
     </row>
     <row r="105">
@@ -4638,7 +4638,7 @@
         <v>0.107</v>
       </c>
       <c r="J105" t="n">
-        <v>0.673</v>
+        <v>0.622</v>
       </c>
     </row>
     <row r="106">
@@ -4678,7 +4678,7 @@
         <v>0.238</v>
       </c>
       <c r="J106" t="n">
-        <v>0.648</v>
+        <v>0.725</v>
       </c>
     </row>
     <row r="107">
@@ -4718,7 +4718,7 @@
         <v>0.238</v>
       </c>
       <c r="J107" t="n">
-        <v>0.836</v>
+        <v>0.772</v>
       </c>
     </row>
     <row r="108">
@@ -4758,7 +4758,7 @@
         <v>0.0919</v>
       </c>
       <c r="J108" t="n">
-        <v>0.0483</v>
+        <v>0.0583</v>
       </c>
     </row>
     <row r="109">
@@ -4878,7 +4878,7 @@
         <v>0.149</v>
       </c>
       <c r="J111" t="n">
-        <v>0.124</v>
+        <v>0.182</v>
       </c>
     </row>
     <row r="112">
@@ -4918,7 +4918,7 @@
         <v>0.18</v>
       </c>
       <c r="J112" t="n">
-        <v>0.0755</v>
+        <v>0.08890000000000001</v>
       </c>
     </row>
     <row r="113">
@@ -4958,7 +4958,7 @@
         <v>0.18</v>
       </c>
       <c r="J113" t="n">
-        <v>0.055</v>
+        <v>0.066</v>
       </c>
     </row>
     <row r="114">
@@ -4998,7 +4998,7 @@
         <v>0.159</v>
       </c>
       <c r="J114" t="n">
-        <v>0.0833</v>
+        <v>0.102</v>
       </c>
     </row>
     <row r="115">
@@ -5038,7 +5038,7 @@
         <v>0.159</v>
       </c>
       <c r="J115" t="n">
-        <v>0.124</v>
+        <v>0.154</v>
       </c>
     </row>
     <row r="116">
@@ -5078,7 +5078,7 @@
         <v>0.161</v>
       </c>
       <c r="J116" t="n">
-        <v>0.107</v>
+        <v>0.154</v>
       </c>
     </row>
     <row r="117">
@@ -5118,7 +5118,7 @@
         <v>0.161</v>
       </c>
       <c r="J117" t="n">
-        <v>0.124</v>
+        <v>0.182</v>
       </c>
     </row>
     <row r="118">
@@ -5158,7 +5158,7 @@
         <v>0.169</v>
       </c>
       <c r="J118" t="n">
-        <v>0.107</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="119">
@@ -5198,7 +5198,7 @@
         <v>0.169</v>
       </c>
       <c r="J119" t="n">
-        <v>0.124</v>
+        <v>0.179</v>
       </c>
     </row>
     <row r="120">
@@ -5238,7 +5238,7 @@
         <v>0.137</v>
       </c>
       <c r="J120" t="n">
-        <v>0.0755</v>
+        <v>0.08890000000000001</v>
       </c>
     </row>
     <row r="121">
@@ -5278,7 +5278,7 @@
         <v>0.137</v>
       </c>
       <c r="J121" t="n">
-        <v>0.055</v>
+        <v>0.0572</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update Table3 and learning curve p-value adjustments
</commit_message>
<xml_diff>
--- a/eval/learning-curve/results/statistical_tests_full150.xlsx
+++ b/eval/learning-curve/results/statistical_tests_full150.xlsx
@@ -518,7 +518,7 @@
         <v>0.102</v>
       </c>
       <c r="J2" t="n">
-        <v>0.319</v>
+        <v>0.195</v>
       </c>
     </row>
     <row r="3">
@@ -558,7 +558,7 @@
         <v>0.102</v>
       </c>
       <c r="J3" t="n">
-        <v>0.334</v>
+        <v>0.2566666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -598,7 +598,7 @@
         <v>0.169</v>
       </c>
       <c r="J4" t="n">
-        <v>0.681</v>
+        <v>0.653</v>
       </c>
     </row>
     <row r="5">
@@ -678,7 +678,7 @@
         <v>0.0877</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="7">
@@ -718,7 +718,7 @@
         <v>0.0877</v>
       </c>
       <c r="J7" t="n">
-        <v>0.495</v>
+        <v>0.335</v>
       </c>
     </row>
     <row r="8">
@@ -758,7 +758,7 @@
         <v>0.156</v>
       </c>
       <c r="J8" t="n">
-        <v>0.755</v>
+        <v>0.653</v>
       </c>
     </row>
     <row r="9">
@@ -798,7 +798,7 @@
         <v>0.156</v>
       </c>
       <c r="J9" t="n">
-        <v>0.765</v>
+        <v>0.80125</v>
       </c>
     </row>
     <row r="10">
@@ -838,7 +838,7 @@
         <v>0.167</v>
       </c>
       <c r="J10" t="n">
-        <v>0.651</v>
+        <v>0.4069999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -878,7 +878,7 @@
         <v>0.167</v>
       </c>
       <c r="J11" t="n">
-        <v>0.773</v>
+        <v>0.6830000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -918,7 +918,7 @@
         <v>0.152</v>
       </c>
       <c r="J12" t="n">
-        <v>0.725</v>
+        <v>0.653</v>
       </c>
     </row>
     <row r="13">
@@ -958,7 +958,7 @@
         <v>0.152</v>
       </c>
       <c r="J13" t="n">
-        <v>0.695</v>
+        <v>0.80125</v>
       </c>
     </row>
     <row r="14">
@@ -998,7 +998,7 @@
         <v>0.0829</v>
       </c>
       <c r="J14" t="n">
-        <v>0.251</v>
+        <v>0.178</v>
       </c>
     </row>
     <row r="15">
@@ -1038,7 +1038,7 @@
         <v>0.0829</v>
       </c>
       <c r="J15" t="n">
-        <v>0.308</v>
+        <v>0.2566666666666667</v>
       </c>
     </row>
     <row r="16">
@@ -1078,7 +1078,7 @@
         <v>0.174</v>
       </c>
       <c r="J16" t="n">
-        <v>0.768</v>
+        <v>0.653</v>
       </c>
     </row>
     <row r="17">
@@ -1118,7 +1118,7 @@
         <v>0.174</v>
       </c>
       <c r="J17" t="n">
-        <v>0.765</v>
+        <v>0.80125</v>
       </c>
     </row>
     <row r="18">
@@ -1158,7 +1158,7 @@
         <v>0.07190000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>0.03</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="19">
@@ -1198,7 +1198,7 @@
         <v>0.07190000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>0.0372</v>
+        <v>0.007299999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -1238,7 +1238,7 @@
         <v>0.0842</v>
       </c>
       <c r="J20" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="21">
@@ -1278,7 +1278,7 @@
         <v>0.0842</v>
       </c>
       <c r="J21" t="n">
-        <v>0.121</v>
+        <v>0.1215</v>
       </c>
     </row>
     <row r="22">
@@ -1318,7 +1318,7 @@
         <v>0.165</v>
       </c>
       <c r="J22" t="n">
-        <v>0.126</v>
+        <v>0.118</v>
       </c>
     </row>
     <row r="23">
@@ -1358,7 +1358,7 @@
         <v>0.165</v>
       </c>
       <c r="J23" t="n">
-        <v>0.123</v>
+        <v>0.1064</v>
       </c>
     </row>
     <row r="24">
@@ -1398,7 +1398,7 @@
         <v>0.175</v>
       </c>
       <c r="J24" t="n">
-        <v>0.395</v>
+        <v>0.3093333333333333</v>
       </c>
     </row>
     <row r="25">
@@ -1438,7 +1438,7 @@
         <v>0.175</v>
       </c>
       <c r="J25" t="n">
-        <v>0.323</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="26">
@@ -1478,7 +1478,7 @@
         <v>0.175</v>
       </c>
       <c r="J26" t="n">
-        <v>0.48</v>
+        <v>0.3093333333333333</v>
       </c>
     </row>
     <row r="27">
@@ -1518,7 +1518,7 @@
         <v>0.175</v>
       </c>
       <c r="J27" t="n">
-        <v>0.495</v>
+        <v>0.339</v>
       </c>
     </row>
     <row r="28">
@@ -1558,7 +1558,7 @@
         <v>0.19</v>
       </c>
       <c r="J28" t="n">
-        <v>0.617</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="29">
@@ -1598,7 +1598,7 @@
         <v>0.19</v>
       </c>
       <c r="J29" t="n">
-        <v>0.598</v>
+        <v>0.339</v>
       </c>
     </row>
     <row r="30">
@@ -1638,7 +1638,7 @@
         <v>0.0931</v>
       </c>
       <c r="J30" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.0144</v>
       </c>
     </row>
     <row r="31">
@@ -1678,7 +1678,7 @@
         <v>0.0931</v>
       </c>
       <c r="J31" t="n">
-        <v>0.0372</v>
+        <v>0.00186</v>
       </c>
     </row>
     <row r="32">
@@ -1718,7 +1718,7 @@
         <v>0.12</v>
       </c>
       <c r="J32" t="n">
-        <v>0.903</v>
+        <v>0.858</v>
       </c>
     </row>
     <row r="33">
@@ -1758,7 +1758,7 @@
         <v>0.12</v>
       </c>
       <c r="J33" t="n">
-        <v>0.634</v>
+        <v>0.4600000000000001</v>
       </c>
     </row>
     <row r="34">
@@ -1798,7 +1798,7 @@
         <v>0.249</v>
       </c>
       <c r="J34" t="n">
-        <v>0.271</v>
+        <v>0.2966666666666666</v>
       </c>
     </row>
     <row r="35">
@@ -1838,7 +1838,7 @@
         <v>0.249</v>
       </c>
       <c r="J35" t="n">
-        <v>0.0572</v>
+        <v>0.03815</v>
       </c>
     </row>
     <row r="36">
@@ -1878,7 +1878,7 @@
         <v>0.134</v>
       </c>
       <c r="J36" t="n">
-        <v>0.768</v>
+        <v>0.858</v>
       </c>
     </row>
     <row r="37">
@@ -1918,7 +1918,7 @@
         <v>0.134</v>
       </c>
       <c r="J37" t="n">
-        <v>0.622</v>
+        <v>0.4600000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -1958,7 +1958,7 @@
         <v>0.22</v>
       </c>
       <c r="J38" t="n">
-        <v>0.581</v>
+        <v>0.3875</v>
       </c>
     </row>
     <row r="39">
@@ -1998,7 +1998,7 @@
         <v>0.22</v>
       </c>
       <c r="J39" t="n">
-        <v>0.447</v>
+        <v>0.28875</v>
       </c>
     </row>
     <row r="40">
@@ -2038,7 +2038,7 @@
         <v>0.185</v>
       </c>
       <c r="J40" t="n">
-        <v>0.395</v>
+        <v>0.4025</v>
       </c>
     </row>
     <row r="41">
@@ -2078,7 +2078,7 @@
         <v>0.185</v>
       </c>
       <c r="J41" t="n">
-        <v>0.179</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="42">
@@ -2118,7 +2118,7 @@
         <v>0.255</v>
       </c>
       <c r="J42" t="n">
-        <v>0.395</v>
+        <v>0.2966666666666666</v>
       </c>
     </row>
     <row r="43">
@@ -2158,7 +2158,7 @@
         <v>0.255</v>
       </c>
       <c r="J43" t="n">
-        <v>0.362</v>
+        <v>0.28875</v>
       </c>
     </row>
     <row r="44">
@@ -2198,7 +2198,7 @@
         <v>0.107</v>
       </c>
       <c r="J44" t="n">
-        <v>0.829</v>
+        <v>0.858</v>
       </c>
     </row>
     <row r="45">
@@ -2238,7 +2238,7 @@
         <v>0.107</v>
       </c>
       <c r="J45" t="n">
-        <v>0.642</v>
+        <v>0.4600000000000001</v>
       </c>
     </row>
     <row r="46">
@@ -2278,7 +2278,7 @@
         <v>0.224</v>
       </c>
       <c r="J46" t="n">
-        <v>0.396</v>
+        <v>0.2966666666666666</v>
       </c>
     </row>
     <row r="47">
@@ -2318,7 +2318,7 @@
         <v>0.224</v>
       </c>
       <c r="J47" t="n">
-        <v>0.222</v>
+        <v>0.18475</v>
       </c>
     </row>
     <row r="48">
@@ -2358,7 +2358,7 @@
         <v>0.0584</v>
       </c>
       <c r="J48" t="n">
-        <v>0.285</v>
+        <v>0.4025</v>
       </c>
     </row>
     <row r="49">
@@ -2398,7 +2398,7 @@
         <v>0.0584</v>
       </c>
       <c r="J49" t="n">
-        <v>0.442</v>
+        <v>0.4600000000000001</v>
       </c>
     </row>
     <row r="50">
@@ -2438,7 +2438,7 @@
         <v>0.11</v>
       </c>
       <c r="J50" t="n">
-        <v>0.883</v>
+        <v>0.8089999999999999</v>
       </c>
     </row>
     <row r="51">
@@ -2478,7 +2478,7 @@
         <v>0.11</v>
       </c>
       <c r="J51" t="n">
-        <v>0.642</v>
+        <v>0.4600000000000001</v>
       </c>
     </row>
     <row r="52">
@@ -2518,7 +2518,7 @@
         <v>0.195</v>
       </c>
       <c r="J52" t="n">
-        <v>0.651</v>
+        <v>0.886</v>
       </c>
     </row>
     <row r="53">
@@ -2558,7 +2558,7 @@
         <v>0.195</v>
       </c>
       <c r="J53" t="n">
-        <v>0.622</v>
+        <v>0.744</v>
       </c>
     </row>
     <row r="54">
@@ -2598,7 +2598,7 @@
         <v>0.183</v>
       </c>
       <c r="J54" t="n">
-        <v>0.917</v>
+        <v>0.886</v>
       </c>
     </row>
     <row r="55">
@@ -2638,7 +2638,7 @@
         <v>0.183</v>
       </c>
       <c r="J55" t="n">
-        <v>0.827</v>
+        <v>0.744</v>
       </c>
     </row>
     <row r="56">
@@ -2678,7 +2678,7 @@
         <v>0.189</v>
       </c>
       <c r="J56" t="n">
-        <v>0.829</v>
+        <v>0.886</v>
       </c>
     </row>
     <row r="57">
@@ -2718,7 +2718,7 @@
         <v>0.189</v>
       </c>
       <c r="J57" t="n">
-        <v>0.765</v>
+        <v>0.744</v>
       </c>
     </row>
     <row r="58">
@@ -2758,7 +2758,7 @@
         <v>0.195</v>
       </c>
       <c r="J58" t="n">
-        <v>0.829</v>
+        <v>0.886</v>
       </c>
     </row>
     <row r="59">
@@ -2798,7 +2798,7 @@
         <v>0.195</v>
       </c>
       <c r="J59" t="n">
-        <v>0.765</v>
+        <v>0.744</v>
       </c>
     </row>
     <row r="60">
@@ -2838,7 +2838,7 @@
         <v>0.0954</v>
       </c>
       <c r="J60" t="n">
-        <v>0.03</v>
+        <v>0.000894</v>
       </c>
     </row>
     <row r="61">
@@ -2878,7 +2878,7 @@
         <v>0.0954</v>
       </c>
       <c r="J61" t="n">
-        <v>0.0372</v>
+        <v>0.000987</v>
       </c>
     </row>
     <row r="62">
@@ -2918,7 +2918,7 @@
         <v>0.186</v>
       </c>
       <c r="J62" t="n">
-        <v>0.54</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="63">
@@ -2958,7 +2958,7 @@
         <v>0.186</v>
       </c>
       <c r="J63" t="n">
-        <v>0.31</v>
+        <v>0.2066666666666667</v>
       </c>
     </row>
     <row r="64">
@@ -3038,7 +3038,7 @@
         <v>0.266</v>
       </c>
       <c r="J65" t="n">
-        <v>0.323</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="66">
@@ -3078,7 +3078,7 @@
         <v>0.149</v>
       </c>
       <c r="J66" t="n">
-        <v>0.755</v>
+        <v>0.592</v>
       </c>
     </row>
     <row r="67">
@@ -3118,7 +3118,7 @@
         <v>0.149</v>
       </c>
       <c r="J67" t="n">
-        <v>0.765</v>
+        <v>0.649</v>
       </c>
     </row>
     <row r="68">
@@ -3158,7 +3158,7 @@
         <v>0.239</v>
       </c>
       <c r="J68" t="n">
-        <v>0.681</v>
+        <v>0.8133333333333334</v>
       </c>
     </row>
     <row r="69">
@@ -3238,7 +3238,7 @@
         <v>0.148</v>
       </c>
       <c r="J70" t="n">
-        <v>0.669</v>
+        <v>0.5575</v>
       </c>
     </row>
     <row r="71">
@@ -3278,7 +3278,7 @@
         <v>0.148</v>
       </c>
       <c r="J71" t="n">
-        <v>0.634</v>
+        <v>0.54125</v>
       </c>
     </row>
     <row r="72">
@@ -3318,7 +3318,7 @@
         <v>0.267</v>
       </c>
       <c r="J72" t="n">
-        <v>0.681</v>
+        <v>0.8133333333333334</v>
       </c>
     </row>
     <row r="73">
@@ -3358,7 +3358,7 @@
         <v>0.267</v>
       </c>
       <c r="J73" t="n">
-        <v>0.895</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -3398,7 +3398,7 @@
         <v>0.144</v>
       </c>
       <c r="J74" t="n">
-        <v>0.347</v>
+        <v>0.3325</v>
       </c>
     </row>
     <row r="75">
@@ -3438,7 +3438,7 @@
         <v>0.144</v>
       </c>
       <c r="J75" t="n">
-        <v>0.308</v>
+        <v>0.2066666666666667</v>
       </c>
     </row>
     <row r="76">
@@ -3478,7 +3478,7 @@
         <v>0.264</v>
       </c>
       <c r="J76" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="77">
@@ -3518,7 +3518,7 @@
         <v>0.264</v>
       </c>
       <c r="J77" t="n">
-        <v>0.622</v>
+        <v>0.605</v>
       </c>
     </row>
     <row r="78">
@@ -3558,7 +3558,7 @@
         <v>0.137</v>
       </c>
       <c r="J78" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.051</v>
       </c>
     </row>
     <row r="79">
@@ -3598,7 +3598,7 @@
         <v>0.137</v>
       </c>
       <c r="J79" t="n">
-        <v>0.066</v>
+        <v>0.05499999999999999</v>
       </c>
     </row>
     <row r="80">
@@ -3638,7 +3638,7 @@
         <v>0.185</v>
       </c>
       <c r="J80" t="n">
-        <v>0.314</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="81">
@@ -3678,7 +3678,7 @@
         <v>0.185</v>
       </c>
       <c r="J81" t="n">
-        <v>0.308</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="82">
@@ -3718,7 +3718,7 @@
         <v>0.18</v>
       </c>
       <c r="J82" t="n">
-        <v>0.09950000000000001</v>
+        <v>0.0199</v>
       </c>
     </row>
     <row r="83">
@@ -3758,7 +3758,7 @@
         <v>0.18</v>
       </c>
       <c r="J83" t="n">
-        <v>0.13</v>
+        <v>0.0303</v>
       </c>
     </row>
     <row r="84">
@@ -3798,7 +3798,7 @@
         <v>0.16</v>
       </c>
       <c r="J84" t="n">
-        <v>0.0583</v>
+        <v>0.01556</v>
       </c>
     </row>
     <row r="85">
@@ -3838,7 +3838,7 @@
         <v>0.16</v>
       </c>
       <c r="J85" t="n">
-        <v>0.0572</v>
+        <v>0.01526</v>
       </c>
     </row>
     <row r="86">
@@ -3878,7 +3878,7 @@
         <v>0.155</v>
       </c>
       <c r="J86" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.0199</v>
       </c>
     </row>
     <row r="87">
@@ -3918,7 +3918,7 @@
         <v>0.155</v>
       </c>
       <c r="J87" t="n">
-        <v>0.109</v>
+        <v>0.02653333333333334</v>
       </c>
     </row>
     <row r="88">
@@ -3958,7 +3958,7 @@
         <v>0.162</v>
       </c>
       <c r="J88" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.0199</v>
       </c>
     </row>
     <row r="89">
@@ -3998,7 +3998,7 @@
         <v>0.162</v>
       </c>
       <c r="J89" t="n">
-        <v>0.0572</v>
+        <v>0.01526</v>
       </c>
     </row>
     <row r="90">
@@ -4038,7 +4038,7 @@
         <v>0.163</v>
       </c>
       <c r="J90" t="n">
-        <v>0.314</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="91">
@@ -4078,7 +4078,7 @@
         <v>0.163</v>
       </c>
       <c r="J91" t="n">
-        <v>0.334</v>
+        <v>0.156</v>
       </c>
     </row>
     <row r="92">
@@ -4118,7 +4118,7 @@
         <v>0.139</v>
       </c>
       <c r="J92" t="n">
-        <v>0.733</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="93">
@@ -4158,7 +4158,7 @@
         <v>0.139</v>
       </c>
       <c r="J93" t="n">
-        <v>0.622</v>
+        <v>0.6733333333333333</v>
       </c>
     </row>
     <row r="94">
@@ -4198,7 +4198,7 @@
         <v>0.247</v>
       </c>
       <c r="J94" t="n">
-        <v>0.651</v>
+        <v>0.5287499999999999</v>
       </c>
     </row>
     <row r="95">
@@ -4238,7 +4238,7 @@
         <v>0.247</v>
       </c>
       <c r="J95" t="n">
-        <v>0.895</v>
+        <v>0.865</v>
       </c>
     </row>
     <row r="96">
@@ -4278,7 +4278,7 @@
         <v>0.116</v>
       </c>
       <c r="J96" t="n">
-        <v>0.903</v>
+        <v>0.8480000000000001</v>
       </c>
     </row>
     <row r="97">
@@ -4318,7 +4318,7 @@
         <v>0.116</v>
       </c>
       <c r="J97" t="n">
-        <v>0.895</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="98">
@@ -4358,7 +4358,7 @@
         <v>0.224</v>
       </c>
       <c r="J98" t="n">
-        <v>0.651</v>
+        <v>0.5287499999999999</v>
       </c>
     </row>
     <row r="99">
@@ -4398,7 +4398,7 @@
         <v>0.224</v>
       </c>
       <c r="J99" t="n">
-        <v>0.895</v>
+        <v>0.865</v>
       </c>
     </row>
     <row r="100">
@@ -4438,7 +4438,7 @@
         <v>0.152</v>
       </c>
       <c r="J100" t="n">
-        <v>0.768</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="101">
@@ -4478,7 +4478,7 @@
         <v>0.152</v>
       </c>
       <c r="J101" t="n">
-        <v>0.765</v>
+        <v>0.8125</v>
       </c>
     </row>
     <row r="102">
@@ -4518,7 +4518,7 @@
         <v>0.256</v>
       </c>
       <c r="J102" t="n">
-        <v>0.616</v>
+        <v>0.5287499999999999</v>
       </c>
     </row>
     <row r="103">
@@ -4558,7 +4558,7 @@
         <v>0.256</v>
       </c>
       <c r="J103" t="n">
-        <v>0.765</v>
+        <v>0.865</v>
       </c>
     </row>
     <row r="104">
@@ -4598,7 +4598,7 @@
         <v>0.107</v>
       </c>
       <c r="J104" t="n">
-        <v>0.616</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="105">
@@ -4638,7 +4638,7 @@
         <v>0.107</v>
       </c>
       <c r="J105" t="n">
-        <v>0.622</v>
+        <v>0.6733333333333333</v>
       </c>
     </row>
     <row r="106">
@@ -4678,7 +4678,7 @@
         <v>0.238</v>
       </c>
       <c r="J106" t="n">
-        <v>0.725</v>
+        <v>0.534</v>
       </c>
     </row>
     <row r="107">
@@ -4718,7 +4718,7 @@
         <v>0.238</v>
       </c>
       <c r="J107" t="n">
-        <v>0.772</v>
+        <v>0.865</v>
       </c>
     </row>
     <row r="108">
@@ -4758,7 +4758,7 @@
         <v>0.0919</v>
       </c>
       <c r="J108" t="n">
-        <v>0.0583</v>
+        <v>0.0161</v>
       </c>
     </row>
     <row r="109">
@@ -4798,7 +4798,7 @@
         <v>0.0919</v>
       </c>
       <c r="J109" t="n">
-        <v>0.0429</v>
+        <v>0.0143</v>
       </c>
     </row>
     <row r="110">
@@ -4838,7 +4838,7 @@
         <v>0.149</v>
       </c>
       <c r="J110" t="n">
-        <v>0.414</v>
+        <v>0.5287499999999999</v>
       </c>
     </row>
     <row r="111">
@@ -4878,7 +4878,7 @@
         <v>0.149</v>
       </c>
       <c r="J111" t="n">
-        <v>0.182</v>
+        <v>0.2885</v>
       </c>
     </row>
     <row r="112">
@@ -4918,7 +4918,7 @@
         <v>0.18</v>
       </c>
       <c r="J112" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.0427</v>
       </c>
     </row>
     <row r="113">
@@ -4958,7 +4958,7 @@
         <v>0.18</v>
       </c>
       <c r="J113" t="n">
-        <v>0.066</v>
+        <v>0.044</v>
       </c>
     </row>
     <row r="114">
@@ -4998,7 +4998,7 @@
         <v>0.159</v>
       </c>
       <c r="J114" t="n">
-        <v>0.102</v>
+        <v>0.0427</v>
       </c>
     </row>
     <row r="115">
@@ -5038,7 +5038,7 @@
         <v>0.159</v>
       </c>
       <c r="J115" t="n">
-        <v>0.154</v>
+        <v>0.0577</v>
       </c>
     </row>
     <row r="116">
@@ -5078,7 +5078,7 @@
         <v>0.161</v>
       </c>
       <c r="J116" t="n">
-        <v>0.154</v>
+        <v>0.0427</v>
       </c>
     </row>
     <row r="117">
@@ -5118,7 +5118,7 @@
         <v>0.161</v>
       </c>
       <c r="J117" t="n">
-        <v>0.182</v>
+        <v>0.0577</v>
       </c>
     </row>
     <row r="118">
@@ -5158,7 +5158,7 @@
         <v>0.169</v>
       </c>
       <c r="J118" t="n">
-        <v>0.16</v>
+        <v>0.0427</v>
       </c>
     </row>
     <row r="119">
@@ -5198,7 +5198,7 @@
         <v>0.169</v>
       </c>
       <c r="J119" t="n">
-        <v>0.179</v>
+        <v>0.0577</v>
       </c>
     </row>
     <row r="120">
@@ -5238,7 +5238,7 @@
         <v>0.137</v>
       </c>
       <c r="J120" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.0151</v>
       </c>
     </row>
     <row r="121">
@@ -5278,7 +5278,7 @@
         <v>0.137</v>
       </c>
       <c r="J121" t="n">
-        <v>0.0572</v>
+        <v>0.0076</v>
       </c>
     </row>
   </sheetData>

</xml_diff>